<commit_message>
add story points to requirements
</commit_message>
<xml_diff>
--- a/documentatie/projectdocumentatie/Requirements.xlsx
+++ b/documentatie/projectdocumentatie/Requirements.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28919"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hrnl-my.sharepoint.com/personal/1079142_hr_nl/Documents/project 78 gedeeld/bestanden/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="595" documentId="8_{D136FF6C-0046-4C4F-AF68-4E782C1807F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0B116AF-1B24-AC48-87CF-663CAF7EFAB9}"/>
+  <xr:revisionPtr revIDLastSave="648" documentId="8_{D136FF6C-0046-4C4F-AF68-4E782C1807F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C12E5708-F870-F34B-8DE7-1FB43F7DA7ED}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{16D86B29-21A7-B547-8524-03D8A703AEA3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="70">
   <si>
     <t>Requirements</t>
   </si>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t>MoSCoW normering</t>
+  </si>
+  <si>
+    <t>Story points</t>
   </si>
   <si>
     <r>
@@ -99,6 +102,67 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1.1.1 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Doe onderzoek naar welke sensoren voldoen aan de gestelde requirements
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1.1.2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Schrijf code die de benodigde data van de radar sensor ophaalt
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">1.1.3 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Implenteer de sensor binnen het prototype</t>
+    </r>
+  </si>
+  <si>
     <t>- er is een sensor die de afstand wordt afgelezen met een nauwkeurigheid van -+ 1cm
 - De sensor is tot op 20 meter afstand nauwkeurig</t>
   </si>
@@ -536,6 +600,47 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">5.1.1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Zet een MQTT broker op om te testen
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">5.1.2 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Zorg ervoor dat de microcontroller via MQTT communiceert.</t>
+    </r>
+  </si>
+  <si>
     <t>- Alle data wordt via mqtt verzonden en komt aan bij de broker</t>
   </si>
   <si>
@@ -801,116 +906,6 @@
     </r>
   </si>
   <si>
-    <t>- Er zit een lcd scherm op waar de afstand, snelheid en status word weergegeven.</t>
-  </si>
-  <si>
-    <t>niet functioneel</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">9. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Het prototype moet een controller bevatten die de data van de sensor leest en met het mqtt netwerk kan verbinden.</t>
-    </r>
-  </si>
-  <si>
-    <t>-De microcontroller maakt verbinding met mqtt en verstuurt sensordata via mqtt</t>
-  </si>
-  <si>
-    <t>versie</t>
-  </si>
-  <si>
-    <t>datum</t>
-  </si>
-  <si>
-    <t>changelog</t>
-  </si>
-  <si>
-    <t>20-02-2025</t>
-  </si>
-  <si>
-    <t>Er is een begin gemaakt aan de requirements.</t>
-  </si>
-  <si>
-    <t>epic=requirement</t>
-  </si>
-  <si>
-    <t>21-02-2025</t>
-  </si>
-  <si>
-    <t>Er is onderscheid gemaakt in functionele en non-functionele requirements en user stories zijn aangevuld.</t>
-  </si>
-  <si>
-    <t>issues=user stories</t>
-  </si>
-  <si>
-    <t>De userstories van requirement 1 zijn verder uitgewerkt. Nu is het sensoronderzoek een aparte user story.</t>
-  </si>
-  <si>
-    <t>Requirement 1 aangepast naar 20 meter ipv 50. 50 is voor een prototype op deze schaal niet realiseerbaar</t>
-  </si>
-  <si>
-    <t>27/03/2025</t>
-  </si>
-  <si>
-    <t>Acceptance criteria bij requirement 9 toegevoegd</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">5.1.1. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Zet een MQTT broker op om te testen
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">5.1.2 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Zorg ervoor dat de microcontroller via MQTT communiceert.</t>
-    </r>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -952,6 +947,33 @@
     </r>
   </si>
   <si>
+    <t>- Er zit een lcd scherm op waar de afstand, snelheid en status word weergegeven.</t>
+  </si>
+  <si>
+    <t>niet functioneel</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">9. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Het prototype moet een controller bevatten die de data van de sensor leest en met het mqtt netwerk kan verbinden.</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -1055,65 +1077,46 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">1.1.1 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Doe onderzoek naar welke sensoren voldoen aan de gestelde requirements
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>1.1.2</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Schrijf code die de benodigde data van de radar sensor ophaalt
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">1.1.3 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Implenteer de sensor binnen het prototype</t>
-    </r>
+    <t>-De microcontroller maakt verbinding met mqtt en verstuurt sensordata via mqtt</t>
+  </si>
+  <si>
+    <t>versie</t>
+  </si>
+  <si>
+    <t>datum</t>
+  </si>
+  <si>
+    <t>changelog</t>
+  </si>
+  <si>
+    <t>20-02-2025</t>
+  </si>
+  <si>
+    <t>Er is een begin gemaakt aan de requirements.</t>
+  </si>
+  <si>
+    <t>epic=requirement</t>
+  </si>
+  <si>
+    <t>21-02-2025</t>
+  </si>
+  <si>
+    <t>Er is onderscheid gemaakt in functionele en non-functionele requirements en user stories zijn aangevuld.</t>
+  </si>
+  <si>
+    <t>issues=user stories</t>
+  </si>
+  <si>
+    <t>De userstories van requirement 1 zijn verder uitgewerkt. Nu is het sensoronderzoek een aparte user story.</t>
+  </si>
+  <si>
+    <t>Requirement 1 aangepast naar 20 meter ipv 50. 50 is voor een prototype op deze schaal niet realiseerbaar</t>
+  </si>
+  <si>
+    <t>27/03/2025</t>
+  </si>
+  <si>
+    <t>Acceptance criteria bij requirement 9 toegevoegd</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1126,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/mm/yy;@"/>
   </numFmts>
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1210,8 +1213,15 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="26"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1245,6 +1255,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1363,7 +1379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1455,9 +1471,6 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1496,6 +1509,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1529,10 +1560,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1865,21 +1892,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{077C9FA5-4E52-DC48-969F-BB8B4D84FDE6}">
   <dimension ref="A1:AP39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
-    <col min="1" max="1" width="63.1640625" customWidth="1"/>
+    <col min="1" max="1" width="63.125" customWidth="1"/>
     <col min="2" max="2" width="36.5" customWidth="1"/>
-    <col min="3" max="3" width="34.6640625" customWidth="1"/>
-    <col min="4" max="4" width="33.83203125" customWidth="1"/>
-    <col min="5" max="5" width="31.6640625" customWidth="1"/>
-    <col min="6" max="6" width="17.83203125" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" customWidth="1"/>
+    <col min="3" max="3" width="34.625" customWidth="1"/>
+    <col min="4" max="4" width="33.875" customWidth="1"/>
+    <col min="5" max="5" width="31.625" customWidth="1"/>
+    <col min="6" max="6" width="17.875" customWidth="1"/>
+    <col min="7" max="7" width="21.5" customWidth="1"/>
+    <col min="8" max="8" width="8.625" customWidth="1"/>
     <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="57" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:42" ht="57" customHeight="1">
       <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
@@ -1895,10 +1922,12 @@
       <c r="E1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="31" t="s">
+      <c r="F1" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1"/>
+      <c r="G1" s="48" t="s">
+        <v>6</v>
+      </c>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="M1" s="2"/>
@@ -1932,26 +1961,28 @@
       <c r="AO1" s="1"/>
       <c r="AP1" s="1"/>
     </row>
-    <row r="2" spans="1:42" ht="115" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:42" ht="114.95" customHeight="1">
       <c r="A2" s="27" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="28" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="26" t="s">
-        <v>68</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="44" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="41" t="s">
+      <c r="D2" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="1"/>
+      <c r="E2" s="43" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="40" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="47">
+        <v>10</v>
+      </c>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="M2" s="2"/>
@@ -1985,18 +2016,20 @@
       <c r="AO2" s="1"/>
       <c r="AP2" s="1"/>
     </row>
-    <row r="3" spans="1:42" ht="130.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:42" ht="130.5" customHeight="1">
       <c r="A3" s="14"/>
       <c r="B3" s="21" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="38"/>
-      <c r="E3" s="44"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="1"/>
+        <v>14</v>
+      </c>
+      <c r="D3" s="37"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="40"/>
+      <c r="G3" s="44">
+        <v>5</v>
+      </c>
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="M3" s="2"/>
@@ -2030,24 +2063,26 @@
       <c r="AO3" s="1"/>
       <c r="AP3" s="1"/>
     </row>
-    <row r="4" spans="1:42" ht="66" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:42" ht="66" customHeight="1">
       <c r="A4" s="20" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B4" s="18" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="42"/>
-      <c r="G4" s="1"/>
+        <v>19</v>
+      </c>
+      <c r="F4" s="41"/>
+      <c r="G4" s="45">
+        <v>4</v>
+      </c>
       <c r="H4" s="2"/>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -2084,26 +2119,28 @@
       <c r="AO4" s="1"/>
       <c r="AP4" s="1"/>
     </row>
-    <row r="5" spans="1:42" ht="117" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:42" ht="117" customHeight="1">
       <c r="A5" s="19" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>22</v>
-      </c>
-      <c r="F5" s="43" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" s="1"/>
+        <v>23</v>
+      </c>
+      <c r="E5" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="42" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="44">
+        <v>5</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -2140,20 +2177,22 @@
       <c r="AO5" s="1"/>
       <c r="AP5" s="1"/>
     </row>
-    <row r="6" spans="1:42" ht="57" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:42" ht="57" customHeight="1">
       <c r="A6" s="11"/>
       <c r="B6" s="12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="40"/>
-      <c r="F6" s="42"/>
-      <c r="G6" s="1"/>
+        <v>27</v>
+      </c>
+      <c r="E6" s="39"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="44">
+        <v>2</v>
+      </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -2190,26 +2229,28 @@
       <c r="AO6" s="1"/>
       <c r="AP6" s="1"/>
     </row>
-    <row r="7" spans="1:42" ht="102" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:42" ht="92.25">
       <c r="A7" s="20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="34" t="s">
-        <v>28</v>
+        <v>29</v>
+      </c>
+      <c r="C7" s="33" t="s">
+        <v>30</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" s="1"/>
+        <v>12</v>
+      </c>
+      <c r="G7" s="46">
+        <v>3</v>
+      </c>
       <c r="H7" s="3"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
@@ -2246,26 +2287,28 @@
       <c r="AO7" s="1"/>
       <c r="AP7" s="1"/>
     </row>
-    <row r="8" spans="1:42" ht="68" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:42" ht="46.5">
       <c r="A8" s="19" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" s="1"/>
+        <v>36</v>
+      </c>
+      <c r="G8" s="44">
+        <v>1</v>
+      </c>
       <c r="H8" s="2"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
@@ -2302,18 +2345,20 @@
       <c r="AO8" s="1"/>
       <c r="AP8" s="1"/>
     </row>
-    <row r="9" spans="1:42" ht="51" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:42" ht="46.5">
       <c r="A9" s="26"/>
       <c r="B9" s="24" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D9" s="8"/>
       <c r="E9" s="9"/>
       <c r="F9" s="17"/>
-      <c r="G9" s="1"/>
+      <c r="G9" s="44">
+        <v>3</v>
+      </c>
       <c r="H9" s="2"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
@@ -2350,26 +2395,28 @@
       <c r="AO9" s="1"/>
       <c r="AP9" s="1"/>
     </row>
-    <row r="10" spans="1:42" ht="53" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:42" ht="53.1" customHeight="1">
       <c r="A10" s="25" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F10" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B10" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="35" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" s="1"/>
+      <c r="G10" s="45">
+        <v>1</v>
+      </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
       <c r="J10" s="2"/>
@@ -2406,26 +2453,28 @@
       <c r="AO10" s="1"/>
       <c r="AP10" s="1"/>
     </row>
-    <row r="11" spans="1:42" ht="117" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:42" ht="117" customHeight="1">
       <c r="A11" s="15" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" s="36" t="s">
-        <v>42</v>
+        <v>44</v>
+      </c>
+      <c r="C11" s="35" t="s">
+        <v>45</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="G11" s="1"/>
+        <v>47</v>
+      </c>
+      <c r="G11" s="44">
+        <v>2</v>
+      </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
@@ -2462,26 +2511,28 @@
       <c r="AO11" s="1"/>
       <c r="AP11" s="1"/>
     </row>
-    <row r="12" spans="1:42" ht="68" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:42" ht="61.5">
       <c r="A12" s="16" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B12" s="22" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C12" s="23" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="D12" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F12" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="F12" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="G12" s="1"/>
+      <c r="G12" s="45">
+        <v>1</v>
+      </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
@@ -2518,26 +2569,28 @@
       <c r="AO12" s="1"/>
       <c r="AP12" s="1"/>
     </row>
-    <row r="13" spans="1:42" ht="170" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:42" ht="138.75">
       <c r="A13" s="21" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>67</v>
+        <v>55</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="G13" s="1"/>
+        <v>36</v>
+      </c>
+      <c r="G13" s="44">
+        <v>4</v>
+      </c>
       <c r="H13" s="1"/>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -2574,7 +2627,7 @@
       <c r="AO13" s="1"/>
       <c r="AP13" s="1"/>
     </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:42">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
@@ -2618,7 +2671,7 @@
       <c r="AO14" s="1"/>
       <c r="AP14" s="1"/>
     </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:42">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="D15" s="1"/>
@@ -2661,15 +2714,15 @@
       <c r="AO15" s="1"/>
       <c r="AP15" s="1"/>
     </row>
-    <row r="16" spans="1:42" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:42" ht="17.100000000000001">
       <c r="A16" s="1" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -2711,19 +2764,19 @@
       <c r="AO16" s="1"/>
       <c r="AP16" s="1"/>
     </row>
-    <row r="17" spans="1:42" ht="34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:42" ht="33.950000000000003">
       <c r="A17" s="1">
         <v>1</v>
       </c>
-      <c r="B17" s="33" t="s">
-        <v>54</v>
+      <c r="B17" s="32" t="s">
+        <v>60</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="D17" s="1"/>
       <c r="E17" s="1" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -2763,19 +2816,19 @@
       <c r="AO17" s="1"/>
       <c r="AP17" s="1"/>
     </row>
-    <row r="18" spans="1:42" ht="51" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:42" ht="51">
       <c r="A18" s="1">
         <v>2</v>
       </c>
-      <c r="B18" s="33" t="s">
-        <v>57</v>
+      <c r="B18" s="32" t="s">
+        <v>63</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D18" s="1"/>
       <c r="E18" s="1" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -2815,15 +2868,15 @@
       <c r="AO18" s="1"/>
       <c r="AP18" s="1"/>
     </row>
-    <row r="19" spans="1:42" ht="51" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:42" ht="51">
       <c r="A19" s="1">
         <v>3</v>
       </c>
-      <c r="B19" s="33">
+      <c r="B19" s="32">
         <v>45723</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
@@ -2865,15 +2918,15 @@
       <c r="AO19" s="1"/>
       <c r="AP19" s="1"/>
     </row>
-    <row r="20" spans="1:42" ht="51" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:42" ht="51">
       <c r="A20" s="1">
         <v>4</v>
       </c>
-      <c r="B20" s="33">
+      <c r="B20" s="32">
         <v>45729</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
@@ -2915,15 +2968,15 @@
       <c r="AO20" s="1"/>
       <c r="AP20" s="1"/>
     </row>
-    <row r="21" spans="1:42" ht="34" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:42" ht="33.950000000000003">
       <c r="A21" s="1">
         <v>5</v>
       </c>
-      <c r="B21" s="32" t="s">
-        <v>62</v>
+      <c r="B21" s="31" t="s">
+        <v>68</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
@@ -2965,9 +3018,9 @@
       <c r="AO21" s="1"/>
       <c r="AP21" s="1"/>
     </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:42">
       <c r="A22" s="1"/>
-      <c r="B22" s="32"/>
+      <c r="B22" s="31"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
@@ -3009,9 +3062,9 @@
       <c r="AO22" s="1"/>
       <c r="AP22" s="1"/>
     </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:42">
       <c r="A23" s="1"/>
-      <c r="B23" s="32"/>
+      <c r="B23" s="31"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
@@ -3053,9 +3106,9 @@
       <c r="AO23" s="1"/>
       <c r="AP23" s="1"/>
     </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:42">
       <c r="A24" s="1"/>
-      <c r="B24" s="32"/>
+      <c r="B24" s="31"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
@@ -3097,9 +3150,9 @@
       <c r="AO24" s="1"/>
       <c r="AP24" s="1"/>
     </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:42">
       <c r="A25" s="1"/>
-      <c r="B25" s="32"/>
+      <c r="B25" s="31"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -3141,9 +3194,9 @@
       <c r="AO25" s="1"/>
       <c r="AP25" s="1"/>
     </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:42">
       <c r="A26" s="1"/>
-      <c r="B26" s="32"/>
+      <c r="B26" s="31"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
@@ -3185,7 +3238,7 @@
       <c r="AO26" s="1"/>
       <c r="AP26" s="1"/>
     </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:42">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
@@ -3229,7 +3282,7 @@
       <c r="AO27" s="1"/>
       <c r="AP27" s="1"/>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:42">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
@@ -3273,7 +3326,7 @@
       <c r="AO28" s="1"/>
       <c r="AP28" s="1"/>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:42">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
@@ -3317,7 +3370,7 @@
       <c r="AO29" s="1"/>
       <c r="AP29" s="1"/>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:42">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
@@ -3361,7 +3414,7 @@
       <c r="AO30" s="1"/>
       <c r="AP30" s="1"/>
     </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:42">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
@@ -3405,7 +3458,7 @@
       <c r="AO31" s="1"/>
       <c r="AP31" s="1"/>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:42">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
@@ -3449,7 +3502,7 @@
       <c r="AO32" s="1"/>
       <c r="AP32" s="1"/>
     </row>
-    <row r="33" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:42">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
@@ -3493,7 +3546,7 @@
       <c r="AO33" s="1"/>
       <c r="AP33" s="1"/>
     </row>
-    <row r="34" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:42">
       <c r="A34" s="1"/>
       <c r="B34" s="1"/>
       <c r="C34" s="1"/>
@@ -3537,7 +3590,7 @@
       <c r="AO34" s="1"/>
       <c r="AP34" s="1"/>
     </row>
-    <row r="35" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:42">
       <c r="A35" s="1"/>
       <c r="B35" s="1"/>
       <c r="C35" s="1"/>
@@ -3581,7 +3634,7 @@
       <c r="AO35" s="1"/>
       <c r="AP35" s="1"/>
     </row>
-    <row r="36" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:42">
       <c r="A36" s="1"/>
       <c r="B36" s="1"/>
       <c r="C36" s="1"/>
@@ -3625,7 +3678,7 @@
       <c r="AO36" s="1"/>
       <c r="AP36" s="1"/>
     </row>
-    <row r="37" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:42">
       <c r="A37" s="1"/>
       <c r="B37" s="1"/>
       <c r="C37" s="1"/>
@@ -3669,7 +3722,7 @@
       <c r="AO37" s="1"/>
       <c r="AP37" s="1"/>
     </row>
-    <row r="38" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:42">
       <c r="A38" s="1"/>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
@@ -3713,7 +3766,7 @@
       <c r="AO38" s="1"/>
       <c r="AP38" s="1"/>
     </row>
-    <row r="39" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:42">
       <c r="A39" s="1"/>
       <c r="B39" s="1"/>
       <c r="C39" s="1"/>

</xml_diff>